<commit_message>
Update BRYT Contract Note estimates spreadsheet
</commit_message>
<xml_diff>
--- a/analysis/BRYT/contract-note/outputs/BRYT Contract Note Estimates.xlsx
+++ b/analysis/BRYT/contract-note/outputs/BRYT Contract Note Estimates.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\d55-analysis\analysis\BRYT\contract-note\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\d55-analysis\analysis\BRYT\contract-note\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A655C16C-2CFC-4101-9505-730687F85C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A967680-2176-4B3E-8AA3-14BAF4371F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Task Detail" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
+    <sheet name="Task Detail" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Task Detail'!$A$1:$F$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Task Detail'!$A$1:$F$136</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="210">
   <si>
     <t>Estimate</t>
   </si>
@@ -1354,15 +1355,15 @@
       </c>
       <c r="C8" s="4">
         <f>SUMIFS('Task Detail'!E:E,'Task Detail'!A:A,A8,'Task Detail'!F:F,"")</f>
-        <v>4.75</v>
+        <v>4.25</v>
       </c>
       <c r="D8" s="4">
         <f>SUMIFS('Task Detail'!E:E,'Task Detail'!A:A,A8,'Task Detail'!F:F,"Yes")</f>
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E8" s="4">
         <f>C8+D8</f>
-        <v>7.75</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
@@ -1396,15 +1397,15 @@
       </c>
       <c r="C10" s="5">
         <f>SUM(C4:C9)</f>
-        <v>40.625</v>
+        <v>40.125</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D4:D9)</f>
-        <v>13</v>
+        <v>12.5</v>
       </c>
       <c r="E10" s="5">
         <f>SUM(E4:E9)</f>
-        <v>53.625</v>
+        <v>52.625</v>
       </c>
     </row>
   </sheetData>
@@ -1416,7 +1417,143 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A837584E-3ED0-4C47-B155-1ABB95CF2FFF}">
+  <dimension ref="A3:E8"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="29.23046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.921875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="13.61328125" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="10.53515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="4">
+        <f>COUNTIF('Task Detail'!A:A,A4)</f>
+        <v>25</v>
+      </c>
+      <c r="C4" s="4">
+        <f>SUMIFS('Task Detail'!E:E,'Task Detail'!A:A,A4,'Task Detail'!F:F,"")</f>
+        <v>4.125</v>
+      </c>
+      <c r="D4" s="4">
+        <f>SUMIFS('Task Detail'!E:E,'Task Detail'!A:A,A4,'Task Detail'!F:F,"Yes")</f>
+        <v>3</v>
+      </c>
+      <c r="E4" s="4">
+        <f>C4+D4</f>
+        <v>7.125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4">
+        <v>7</v>
+      </c>
+      <c r="C5" s="4">
+        <v>4</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4">
+        <f>COUNTIF('Task Detail'!A:A,A6)</f>
+        <v>26</v>
+      </c>
+      <c r="C6" s="4">
+        <f>SUMIFS('Task Detail'!E:E,'Task Detail'!A:A,A6,'Task Detail'!F:F,"")</f>
+        <v>6.375</v>
+      </c>
+      <c r="D6" s="4">
+        <f>SUMIFS('Task Detail'!E:E,'Task Detail'!A:A,A6,'Task Detail'!F:F,"Yes")</f>
+        <v>2.5</v>
+      </c>
+      <c r="E6" s="4">
+        <f>C6+D6</f>
+        <v>8.875</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4">
+        <f>COUNTIF('Task Detail'!A:A,A7)</f>
+        <v>25</v>
+      </c>
+      <c r="C7" s="4">
+        <f>SUMIFS('Task Detail'!E:E,'Task Detail'!A:A,A7,'Task Detail'!F:F,"")</f>
+        <v>4.25</v>
+      </c>
+      <c r="D7" s="4">
+        <f>SUMIFS('Task Detail'!E:E,'Task Detail'!A:A,A7,'Task Detail'!F:F,"Yes")</f>
+        <v>2.5</v>
+      </c>
+      <c r="E7" s="4">
+        <f>C7+D7</f>
+        <v>6.75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="5">
+        <f>SUM(B4:B7)</f>
+        <v>83</v>
+      </c>
+      <c r="C8" s="5">
+        <f>SUM(C4:C7)</f>
+        <v>18.75</v>
+      </c>
+      <c r="D8" s="5">
+        <f>SUM(D4:D7)</f>
+        <v>8</v>
+      </c>
+      <c r="E8" s="5">
+        <f>SUM(E4:E7)</f>
+        <v>26.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F136"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
@@ -1448,7 +1585,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
@@ -1466,7 +1603,7 @@
       </c>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
@@ -1484,7 +1621,7 @@
       </c>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
@@ -1502,7 +1639,7 @@
       </c>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
@@ -1522,7 +1659,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
@@ -1540,7 +1677,7 @@
       </c>
       <c r="F6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
@@ -1558,7 +1695,7 @@
       </c>
       <c r="F7" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A8" s="6" t="s">
         <v>5</v>
       </c>
@@ -1576,7 +1713,7 @@
       </c>
       <c r="F8" s="2"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A9" s="6" t="s">
         <v>5</v>
       </c>
@@ -1594,7 +1731,7 @@
       </c>
       <c r="F9" s="2"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
         <v>5</v>
       </c>
@@ -1612,7 +1749,7 @@
       </c>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A11" s="6" t="s">
         <v>5</v>
       </c>
@@ -1630,7 +1767,7 @@
       </c>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A12" s="6" t="s">
         <v>5</v>
       </c>
@@ -1650,7 +1787,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A13" s="6" t="s">
         <v>5</v>
       </c>
@@ -1668,7 +1805,7 @@
       </c>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A14" s="6" t="s">
         <v>5</v>
       </c>
@@ -1686,7 +1823,7 @@
       </c>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" s="6" t="s">
         <v>5</v>
       </c>
@@ -1704,7 +1841,7 @@
       </c>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>5</v>
       </c>
@@ -1722,7 +1859,7 @@
       </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A17" s="6" t="s">
         <v>5</v>
       </c>
@@ -1740,7 +1877,7 @@
       </c>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A18" s="6" t="s">
         <v>5</v>
       </c>
@@ -1758,7 +1895,7 @@
       </c>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A19" s="6" t="s">
         <v>5</v>
       </c>
@@ -1776,7 +1913,7 @@
       </c>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A20" s="6" t="s">
         <v>5</v>
       </c>
@@ -1794,7 +1931,7 @@
       </c>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
         <v>5</v>
       </c>
@@ -1814,7 +1951,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A22" s="6" t="s">
         <v>5</v>
       </c>
@@ -1832,7 +1969,7 @@
       </c>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A23" s="6" t="s">
         <v>5</v>
       </c>
@@ -1850,7 +1987,7 @@
       </c>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A24" s="6" t="s">
         <v>5</v>
       </c>
@@ -1868,7 +2005,7 @@
       </c>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A25" s="6" t="s">
         <v>5</v>
       </c>
@@ -1888,7 +2025,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A26" s="6" t="s">
         <v>5</v>
       </c>
@@ -1906,7 +2043,7 @@
       </c>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A27" s="6" t="s">
         <v>5</v>
       </c>
@@ -1924,7 +2061,7 @@
       </c>
       <c r="F27" s="2"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A28" s="6" t="s">
         <v>5</v>
       </c>
@@ -1944,7 +2081,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A29" s="6" t="s">
         <v>5</v>
       </c>
@@ -1962,7 +2099,7 @@
       </c>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A30" s="6" t="s">
         <v>5</v>
       </c>
@@ -1982,7 +2119,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A31" s="6" t="s">
         <v>5</v>
       </c>
@@ -2000,7 +2137,7 @@
       </c>
       <c r="F31" s="2"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A32" s="6" t="s">
         <v>5</v>
       </c>
@@ -2020,7 +2157,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A33" s="6" t="s">
         <v>5</v>
       </c>
@@ -2038,7 +2175,7 @@
       </c>
       <c r="F33" s="2"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A34" s="6" t="s">
         <v>5</v>
       </c>
@@ -2056,7 +2193,7 @@
       </c>
       <c r="F34" s="2"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A35" s="6" t="s">
         <v>5</v>
       </c>
@@ -2074,7 +2211,7 @@
       </c>
       <c r="F35" s="2"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A36" s="6" t="s">
         <v>5</v>
       </c>
@@ -2092,7 +2229,7 @@
       </c>
       <c r="F36" s="2"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A37" s="6" t="s">
         <v>5</v>
       </c>
@@ -2110,7 +2247,7 @@
       </c>
       <c r="F37" s="2"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A38" s="6" t="s">
         <v>5</v>
       </c>
@@ -2128,7 +2265,7 @@
       </c>
       <c r="F38" s="2"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A39" s="6" t="s">
         <v>5</v>
       </c>
@@ -2146,7 +2283,7 @@
       </c>
       <c r="F39" s="2"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A40" s="6" t="s">
         <v>5</v>
       </c>
@@ -2164,7 +2301,7 @@
       </c>
       <c r="F40" s="2"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A41" s="6" t="s">
         <v>5</v>
       </c>
@@ -2184,7 +2321,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A42" s="6" t="s">
         <v>5</v>
       </c>
@@ -2202,7 +2339,7 @@
       </c>
       <c r="F42" s="2"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A43" s="6" t="s">
         <v>5</v>
       </c>
@@ -2220,7 +2357,7 @@
       </c>
       <c r="F43" s="2"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A44" s="6" t="s">
         <v>5</v>
       </c>
@@ -3230,7 +3367,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="2">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>28</v>
@@ -3358,7 +3495,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="2">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="F105" s="2" t="s">
         <v>28</v>
@@ -3600,7 +3737,7 @@
         <v>19</v>
       </c>
       <c r="E118" s="2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F118" s="2"/>
     </row>
@@ -3931,7 +4068,16 @@
       <c r="F136" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F136" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:F136" xr:uid="{00000000-0009-0000-0000-000001000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Est 2: DocuSign Integration"/>
+        <filter val="Est 3b: Data Source Extensibility"/>
+        <filter val="Est 4: Bespoke Contracts"/>
+        <filter val="Est 5: Comparison Audit"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="D2:D136">
     <cfRule type="cellIs" dxfId="10" priority="6" operator="equal">
       <formula>"prompt_iteration"</formula>

</xml_diff>